<commit_message>
sprint 5 review, checklists eklendi, gant chart düzenlendi
</commit_message>
<xml_diff>
--- a/Docs/Gant Chart.xlsx
+++ b/Docs/Gant Chart.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="26">
   <si>
     <t>Görev</t>
   </si>
@@ -43,40 +43,46 @@
     <t>Tamamlandı</t>
   </si>
   <si>
-    <t>Testlerin planlanması ve senaryolaştırılması ve "Test Document v1.0" teslimi</t>
+    <t>QMP v1.0</t>
   </si>
   <si>
     <t>Kerem ELMA</t>
   </si>
   <si>
-    <t>Design document güncellenecek</t>
+    <t>Final System Architecture Diagram tasarlanacak</t>
+  </si>
+  <si>
+    <t>Final Quality model teslim edilecek</t>
   </si>
   <si>
     <t>Mete Cem TURAN</t>
   </si>
   <si>
-    <t>Quality metriklerinin oluşturulması</t>
+    <t>Define quality measurements and metrics for all target features</t>
+  </si>
+  <si>
+    <t>Mehmet ESKİ</t>
+  </si>
+  <si>
+    <t>Project Management Plan v2.0(PMP)</t>
   </si>
   <si>
     <t>Sabri Mert PİŞKİN</t>
   </si>
   <si>
-    <t>Unit, integration ve system test'lerinin nasıl çalışacağına karar verilmesi</t>
-  </si>
-  <si>
-    <t>Mehmet ESKİ</t>
-  </si>
-  <si>
-    <t>Sequence, State Machine, Deployment Diagram hazırlanması</t>
-  </si>
-  <si>
-    <t>Sprint 4 Review</t>
-  </si>
-  <si>
-    <t>Trello ve Github ortamında issue tanımlamaları ve takipleri</t>
+    <t>Project Management Plan oluşturulacak</t>
+  </si>
+  <si>
+    <t>SRS + Design + Test + Technology Comparison Report yeni template varsa güncellenecek</t>
   </si>
   <si>
     <t>Trello ortamında issue tanımlamaları ve takipleri</t>
+  </si>
+  <si>
+    <t>Proje Kontrol Listesi v2</t>
+  </si>
+  <si>
+    <t>Sprint 5 Review</t>
   </si>
   <si>
     <t>Yapılacak</t>
@@ -135,7 +141,7 @@
       <name val="Roboto"/>
     </font>
     <font>
-      <color rgb="FF5A3286"/>
+      <color rgb="FF000000"/>
       <name val="Roboto"/>
     </font>
     <font>
@@ -144,11 +150,13 @@
       <name val="'Times New Roman'"/>
     </font>
     <font>
-      <color rgb="FF000000"/>
-      <name val="Roboto"/>
+      <color rgb="FF0A53A8"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <color rgb="FF0A53A8"/>
+      <sz val="100.0"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -203,7 +211,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border/>
     <border>
       <left style="thin">
@@ -241,22 +249,11 @@
         <color rgb="FFFFFFFF"/>
       </top>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFFFFFFF"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF284E3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFFFFFFF"/>
-      </top>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -291,9 +288,6 @@
     <xf borderId="1" fillId="4" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="2" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="3" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="3" fillId="4" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -302,42 +296,45 @@
     <xf borderId="3" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="4" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf borderId="1" fillId="5" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="6" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="1" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="6" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="6" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="8" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="4" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -417,7 +414,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:F9" displayName="Tablo1" name="Tablo1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:F11" displayName="Tablo1" name="Tablo1" id="1">
   <tableColumns count="6">
     <tableColumn name="Görev" id="1"/>
     <tableColumn name="Kim" id="2"/>
@@ -431,8 +428,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="H2:V14" displayName="Table_1" name="Table_1" id="2">
-  <tableColumns count="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="H2:U17" displayName="Table_1" name="Table_1" id="2">
+  <tableColumns count="14">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
     <tableColumn name="Column3" id="3"/>
@@ -447,7 +444,6 @@
     <tableColumn name="Column12" id="12"/>
     <tableColumn name="Column13" id="13"/>
     <tableColumn name="Column14" id="14"/>
-    <tableColumn name="Column15" id="15"/>
   </tableColumns>
   <tableStyleInfo name="Sayfa1-style 2" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
@@ -654,13 +650,13 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="59.75"/>
+    <col customWidth="1" min="1" max="1" width="69.5"/>
     <col customWidth="1" min="2" max="2" width="15.63"/>
     <col customWidth="1" min="3" max="3" width="20.5"/>
     <col customWidth="1" min="4" max="4" width="13.25"/>
     <col customWidth="1" min="5" max="5" width="13.38"/>
     <col customWidth="1" min="6" max="6" width="13.75"/>
-    <col customWidth="1" min="8" max="8" width="59.13"/>
+    <col customWidth="1" min="8" max="8" width="72.63"/>
     <col customWidth="1" min="9" max="9" width="3.25"/>
     <col customWidth="1" min="10" max="10" width="3.38"/>
     <col customWidth="1" min="11" max="11" width="3.25"/>
@@ -669,16 +665,14 @@
     <col customWidth="1" min="14" max="14" width="3.0"/>
     <col customWidth="1" min="15" max="15" width="2.88"/>
     <col customWidth="1" min="16" max="16" width="3.13"/>
-    <col customWidth="1" min="17" max="17" width="2.88"/>
-    <col customWidth="1" min="18" max="18" width="3.25"/>
-    <col customWidth="1" min="19" max="19" width="2.88"/>
-    <col customWidth="1" min="20" max="20" width="3.0"/>
-    <col customWidth="1" min="21" max="21" width="3.25"/>
-    <col customWidth="1" min="22" max="22" width="3.0"/>
-    <col customWidth="1" min="23" max="23" width="4.13"/>
-    <col customWidth="1" min="24" max="24" width="4.25"/>
-    <col customWidth="1" min="25" max="25" width="5.0"/>
-    <col customWidth="1" min="26" max="26" width="4.63"/>
+    <col customWidth="1" min="17" max="18" width="2.88"/>
+    <col customWidth="1" min="19" max="19" width="3.0"/>
+    <col customWidth="1" min="20" max="20" width="3.25"/>
+    <col customWidth="1" min="21" max="21" width="3.0"/>
+    <col customWidth="1" min="22" max="22" width="4.13"/>
+    <col customWidth="1" min="23" max="23" width="4.25"/>
+    <col customWidth="1" min="24" max="24" width="5.0"/>
+    <col customWidth="1" min="25" max="25" width="4.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
@@ -704,37 +698,42 @@
         <v>6</v>
       </c>
       <c r="I1" s="4">
-        <v>25.0</v>
+        <v>6.0</v>
       </c>
       <c r="J1" s="4">
-        <v>26.0</v>
+        <v>7.0</v>
       </c>
       <c r="K1" s="4">
-        <v>27.0</v>
+        <v>8.0</v>
       </c>
       <c r="L1" s="4">
-        <v>28.0</v>
+        <v>9.0</v>
       </c>
       <c r="M1" s="4">
-        <v>29.0</v>
+        <v>10.0</v>
       </c>
       <c r="N1" s="4">
-        <v>30.0</v>
+        <v>11.0</v>
       </c>
       <c r="O1" s="4">
-        <v>1.0</v>
+        <v>12.0</v>
       </c>
       <c r="P1" s="4">
-        <v>2.0</v>
+        <v>13.0</v>
       </c>
       <c r="Q1" s="4">
-        <v>3.0</v>
-      </c>
-      <c r="R1" s="5"/>
-      <c r="S1" s="5"/>
-      <c r="T1" s="5"/>
+        <v>14.0</v>
+      </c>
+      <c r="R1" s="4">
+        <v>15.0</v>
+      </c>
+      <c r="S1" s="4">
+        <v>16.0</v>
+      </c>
+      <c r="T1" s="4">
+        <v>17.0</v>
+      </c>
       <c r="U1" s="5"/>
-      <c r="V1" s="5"/>
     </row>
     <row r="2" ht="18.75" customHeight="1">
       <c r="A2" s="6" t="s">
@@ -744,10 +743,10 @@
         <v>8</v>
       </c>
       <c r="C2" s="7">
-        <v>45986.0</v>
+        <v>45997.0</v>
       </c>
       <c r="D2" s="7">
-        <v>45986.0</v>
+        <v>45997.0</v>
       </c>
       <c r="E2" s="6">
         <v>1.0</v>
@@ -760,17 +759,17 @@
       </c>
       <c r="I2" s="10"/>
       <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
       <c r="L2" s="11"/>
       <c r="M2" s="11"/>
       <c r="N2" s="11"/>
       <c r="O2" s="11"/>
       <c r="P2" s="11"/>
       <c r="Q2" s="11"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12"/>
-      <c r="T2" s="12"/>
+      <c r="R2" s="11"/>
+      <c r="S2" s="11"/>
+      <c r="T2" s="11"/>
       <c r="U2" s="12"/>
-      <c r="V2" s="12"/>
     </row>
     <row r="3" ht="19.5" customHeight="1">
       <c r="A3" s="6" t="s">
@@ -780,13 +779,13 @@
         <v>11</v>
       </c>
       <c r="C3" s="7">
-        <v>45989.0</v>
+        <v>46000.0</v>
       </c>
       <c r="D3" s="7">
-        <v>45990.0</v>
+        <v>46002.0</v>
       </c>
       <c r="E3" s="6">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="F3" s="8" t="s">
         <v>9</v>
@@ -799,31 +798,30 @@
       <c r="K3" s="11"/>
       <c r="L3" s="10"/>
       <c r="M3" s="10"/>
-      <c r="N3" s="11"/>
+      <c r="N3" s="10"/>
       <c r="O3" s="11"/>
       <c r="P3" s="11"/>
       <c r="Q3" s="11"/>
-      <c r="R3" s="12"/>
-      <c r="S3" s="12"/>
-      <c r="T3" s="12"/>
+      <c r="R3" s="11"/>
+      <c r="S3" s="11"/>
+      <c r="T3" s="11"/>
       <c r="U3" s="12"/>
-      <c r="V3" s="12"/>
     </row>
     <row r="4" ht="18.0" customHeight="1">
       <c r="A4" s="6" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C4" s="7">
-        <v>45989.0</v>
+        <v>46000.0</v>
       </c>
       <c r="D4" s="7">
-        <v>45990.0</v>
+        <v>46002.0</v>
       </c>
       <c r="E4" s="6">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="F4" s="8" t="s">
         <v>9</v>
@@ -836,28 +834,27 @@
       <c r="K4" s="11"/>
       <c r="L4" s="10"/>
       <c r="M4" s="10"/>
-      <c r="N4" s="11"/>
+      <c r="N4" s="10"/>
       <c r="O4" s="11"/>
       <c r="P4" s="11"/>
       <c r="Q4" s="11"/>
-      <c r="R4" s="12"/>
-      <c r="S4" s="12"/>
-      <c r="T4" s="12"/>
+      <c r="R4" s="11"/>
+      <c r="S4" s="11"/>
+      <c r="T4" s="11"/>
       <c r="U4" s="12"/>
-      <c r="V4" s="12"/>
     </row>
     <row r="5" ht="16.5" customHeight="1">
       <c r="A5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>15</v>
-      </c>
       <c r="C5" s="7">
-        <v>45989.0</v>
+        <v>46000.0</v>
       </c>
       <c r="D5" s="7">
-        <v>45991.0</v>
+        <v>46002.0</v>
       </c>
       <c r="E5" s="6">
         <v>3.0</v>
@@ -866,7 +863,7 @@
         <v>9</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I5" s="11"/>
       <c r="J5" s="11"/>
@@ -877,212 +874,237 @@
       <c r="O5" s="11"/>
       <c r="P5" s="11"/>
       <c r="Q5" s="11"/>
-      <c r="R5" s="12"/>
-      <c r="S5" s="12"/>
-      <c r="T5" s="12"/>
+      <c r="R5" s="11"/>
+      <c r="S5" s="11"/>
+      <c r="T5" s="11"/>
       <c r="U5" s="12"/>
-      <c r="V5" s="12"/>
-    </row>
-    <row r="6" ht="16.5" customHeight="1">
-      <c r="A6" s="6" t="s">
+    </row>
+    <row r="6" ht="17.25" customHeight="1">
+      <c r="A6" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="7">
-        <v>45992.0</v>
+      <c r="C6" s="14">
+        <v>46001.0</v>
       </c>
       <c r="D6" s="7">
-        <v>45993.0</v>
-      </c>
-      <c r="E6" s="6">
-        <v>2.0</v>
+        <v>46004.0</v>
+      </c>
+      <c r="E6" s="15">
+        <v>4.0</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="9" t="s">
-        <v>16</v>
+      <c r="H6" s="16" t="s">
+        <v>15</v>
       </c>
       <c r="I6" s="11"/>
       <c r="J6" s="11"/>
       <c r="K6" s="11"/>
       <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
       <c r="O6" s="10"/>
       <c r="P6" s="10"/>
       <c r="Q6" s="11"/>
-      <c r="R6" s="12"/>
-      <c r="S6" s="12"/>
-      <c r="T6" s="12"/>
+      <c r="R6" s="11"/>
+      <c r="S6" s="11"/>
+      <c r="T6" s="11"/>
       <c r="U6" s="12"/>
-      <c r="V6" s="12"/>
     </row>
     <row r="7" ht="17.25" customHeight="1">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="15">
-        <v>45989.0</v>
-      </c>
-      <c r="D7" s="15">
-        <v>45993.0</v>
-      </c>
-      <c r="E7" s="16">
-        <v>4.0</v>
-      </c>
-      <c r="F7" s="17" t="s">
+      <c r="C7" s="7">
+        <v>46006.0</v>
+      </c>
+      <c r="D7" s="7">
+        <v>46008.0</v>
+      </c>
+      <c r="E7" s="18">
+        <v>2.0</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="H7" s="9" t="s">
-        <v>18</v>
+      <c r="H7" s="16" t="s">
+        <v>19</v>
       </c>
       <c r="I7" s="11"/>
       <c r="J7" s="11"/>
       <c r="K7" s="11"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10"/>
-      <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
-      <c r="Q7" s="11"/>
-      <c r="R7" s="12"/>
-      <c r="S7" s="12"/>
-      <c r="T7" s="12"/>
+      <c r="L7" s="11"/>
+      <c r="M7" s="11"/>
+      <c r="N7" s="11"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="19"/>
+      <c r="Q7" s="19"/>
+      <c r="R7" s="10"/>
+      <c r="S7" s="10"/>
+      <c r="T7" s="11"/>
       <c r="U7" s="12"/>
-      <c r="V7" s="12"/>
-    </row>
-    <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="19">
-        <v>45994.0</v>
-      </c>
-      <c r="D8" s="19">
-        <v>45994.0</v>
-      </c>
-      <c r="E8" s="20">
-        <v>1.0</v>
-      </c>
-      <c r="F8" s="21" t="s">
+    </row>
+    <row r="8" ht="17.25" customHeight="1">
+      <c r="A8" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="7">
+        <v>46006.0</v>
+      </c>
+      <c r="D8" s="14">
+        <v>46008.0</v>
+      </c>
+      <c r="E8" s="18">
+        <v>2.0</v>
+      </c>
+      <c r="F8" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="H8" s="9" t="s">
-        <v>19</v>
+      <c r="H8" s="16" t="s">
+        <v>20</v>
       </c>
       <c r="I8" s="11"/>
       <c r="J8" s="11"/>
       <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
       <c r="N8" s="11"/>
       <c r="O8" s="11"/>
       <c r="P8" s="11"/>
-      <c r="Q8" s="10"/>
-      <c r="R8" s="12"/>
-      <c r="S8" s="12"/>
-      <c r="T8" s="12"/>
+      <c r="Q8" s="19"/>
+      <c r="R8" s="10"/>
+      <c r="S8" s="10"/>
+      <c r="T8" s="11"/>
       <c r="U8" s="12"/>
-      <c r="V8" s="12"/>
-    </row>
-    <row r="9" ht="18.0" customHeight="1">
+    </row>
+    <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="19">
-        <v>45986.0</v>
-      </c>
-      <c r="D9" s="19">
-        <v>45994.0</v>
-      </c>
-      <c r="E9" s="20">
-        <v>9.0</v>
-      </c>
-      <c r="F9" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="20">
+        <v>45997.0</v>
+      </c>
+      <c r="D9" s="7">
+        <v>46004.0</v>
+      </c>
+      <c r="E9" s="18">
+        <v>8.0</v>
+      </c>
+      <c r="F9" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="G9" s="22"/>
       <c r="H9" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
       <c r="L9" s="10"/>
       <c r="M9" s="10"/>
       <c r="N9" s="10"/>
       <c r="O9" s="10"/>
       <c r="P9" s="10"/>
-      <c r="Q9" s="10"/>
-      <c r="R9" s="12"/>
-      <c r="S9" s="12"/>
-      <c r="T9" s="12"/>
+      <c r="Q9" s="11"/>
+      <c r="R9" s="11"/>
+      <c r="S9" s="11"/>
+      <c r="T9" s="11"/>
       <c r="U9" s="12"/>
-      <c r="V9" s="12"/>
-    </row>
-    <row r="10">
-      <c r="G10" s="22"/>
-      <c r="H10" s="23"/>
-      <c r="N10" s="12"/>
-      <c r="O10" s="12"/>
-      <c r="P10" s="12"/>
-      <c r="Q10" s="12"/>
-      <c r="R10" s="12"/>
-      <c r="S10" s="12"/>
-      <c r="T10" s="12"/>
+    </row>
+    <row r="10" ht="18.0" customHeight="1">
+      <c r="A10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="20">
+        <v>46008.0</v>
+      </c>
+      <c r="D10" s="20">
+        <v>46008.0</v>
+      </c>
+      <c r="E10" s="18">
+        <v>1.0</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10" s="21"/>
+      <c r="H10" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="I10" s="11"/>
+      <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="11"/>
+      <c r="M10" s="11"/>
+      <c r="N10" s="11"/>
+      <c r="O10" s="11"/>
+      <c r="P10" s="11"/>
+      <c r="Q10" s="11"/>
+      <c r="R10" s="11"/>
+      <c r="S10" s="11"/>
+      <c r="T10" s="10"/>
       <c r="U10" s="12"/>
-      <c r="V10" s="12"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="24"/>
-      <c r="B11" s="24"/>
-      <c r="C11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="27" t="s">
-        <v>22</v>
-      </c>
-      <c r="K11" s="28"/>
-      <c r="L11" s="28"/>
-      <c r="M11" s="29"/>
-      <c r="N11" s="12"/>
-      <c r="O11" s="12"/>
-      <c r="P11" s="12"/>
-      <c r="Q11" s="12"/>
-      <c r="R11" s="12"/>
-      <c r="S11" s="12"/>
-      <c r="T11" s="12"/>
+    </row>
+    <row r="11" ht="20.25" customHeight="1">
+      <c r="A11" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="20">
+        <v>46008.0</v>
+      </c>
+      <c r="D11" s="20">
+        <v>46008.0</v>
+      </c>
+      <c r="E11" s="18">
+        <v>1.0</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G11" s="21"/>
+      <c r="H11" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="11"/>
+      <c r="M11" s="11"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="11"/>
+      <c r="P11" s="11"/>
+      <c r="Q11" s="11"/>
+      <c r="R11" s="11"/>
+      <c r="S11" s="11"/>
+      <c r="T11" s="10"/>
       <c r="U11" s="12"/>
-      <c r="V11" s="12"/>
     </row>
     <row r="12">
-      <c r="A12" s="24"/>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="E12" s="24"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="27" t="s">
-        <v>9</v>
-      </c>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="12"/>
+      <c r="A12" s="22"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="23"/>
+      <c r="M12" s="24"/>
       <c r="N12" s="12"/>
       <c r="O12" s="12"/>
       <c r="P12" s="12"/>
@@ -1091,94 +1113,134 @@
       <c r="S12" s="12"/>
       <c r="T12" s="12"/>
       <c r="U12" s="12"/>
-      <c r="V12" s="12"/>
     </row>
     <row r="13">
-      <c r="A13" s="24"/>
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="E13" s="24"/>
+      <c r="A13" s="22"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="G13" s="21"/>
       <c r="H13" s="23"/>
-      <c r="I13" s="30"/>
-      <c r="J13" s="27" t="s">
-        <v>23</v>
-      </c>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
       <c r="M13" s="12"/>
-      <c r="N13" s="29"/>
-      <c r="O13" s="29"/>
-      <c r="P13" s="29"/>
-      <c r="Q13" s="29"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="12"/>
+      <c r="Q13" s="12"/>
       <c r="R13" s="12"/>
       <c r="S13" s="12"/>
       <c r="T13" s="12"/>
       <c r="U13" s="12"/>
-      <c r="V13" s="12"/>
     </row>
     <row r="14">
-      <c r="A14" s="24"/>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="H14" s="31"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="12"/>
+      <c r="A14" s="22"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="H14" s="25"/>
       <c r="M14" s="12"/>
-      <c r="N14" s="12"/>
-      <c r="O14" s="12"/>
-      <c r="P14" s="12"/>
-      <c r="Q14" s="12"/>
-      <c r="R14" s="29"/>
-      <c r="S14" s="29"/>
-      <c r="T14" s="29"/>
-      <c r="U14" s="29"/>
-      <c r="V14" s="29"/>
+      <c r="N14" s="24"/>
+      <c r="O14" s="24"/>
+      <c r="P14" s="24"/>
+      <c r="Q14" s="24"/>
+      <c r="R14" s="12"/>
+      <c r="S14" s="12"/>
+      <c r="T14" s="12"/>
+      <c r="U14" s="12"/>
     </row>
     <row r="15">
-      <c r="A15" s="24"/>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="H15" s="32"/>
+      <c r="A15" s="22"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="K15" s="29"/>
+      <c r="L15" s="29"/>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12"/>
+      <c r="O15" s="12"/>
+      <c r="P15" s="12"/>
+      <c r="Q15" s="12"/>
+      <c r="R15" s="24"/>
+      <c r="S15" s="24"/>
+      <c r="T15" s="24"/>
+      <c r="U15" s="24"/>
     </row>
     <row r="16">
-      <c r="A16" s="24"/>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="H16" s="32"/>
+      <c r="A16" s="22"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="H16" s="30"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="K16" s="11"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="31"/>
+      <c r="N16" s="31"/>
+      <c r="O16" s="31"/>
+      <c r="P16" s="31"/>
+      <c r="Q16" s="31"/>
+      <c r="R16" s="24"/>
+      <c r="S16" s="24"/>
+      <c r="T16" s="24"/>
+      <c r="U16" s="24"/>
     </row>
     <row r="17">
-      <c r="A17" s="24"/>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="H17" s="32"/>
+      <c r="A17" s="22"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="22"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="33"/>
+      <c r="J17" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11"/>
+      <c r="M17" s="31"/>
+      <c r="N17" s="31"/>
+      <c r="O17" s="31"/>
+      <c r="P17" s="31"/>
+      <c r="Q17" s="31"/>
+      <c r="R17" s="24"/>
+      <c r="S17" s="24"/>
+      <c r="T17" s="24"/>
+      <c r="U17" s="24"/>
     </row>
     <row r="18">
-      <c r="A18" s="24"/>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
+      <c r="A18" s="22"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="H18" s="34"/>
     </row>
     <row r="19">
-      <c r="A19" s="24"/>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
+      <c r="A19" s="22"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="22"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="C2:C9">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="C2:C11">
       <formula1>OR(NOT(ISERROR(DATEVALUE(C2))), AND(ISNUMBER(C2), LEFT(CELL("format", C2))="D"))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F9">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F11">
       <formula1>"Tamamlandı,Yapılacak,Devam Ediyor"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>